<commit_message>
Migrate Deluxe homepage to EDS
Add block variants (cards-product, cards-news, cards-services,
story-banner, tabs-solutions), rebuilt cards-stats, Deluxe nav/footer,
design system styles, and import tooling (parsers, transformers,
page templates). Include imported homepage content and brand assets.
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -40,7 +40,7 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["hero-video","carousel-spotlight","accordion-pillars","tabs-casestudy","tabs-casestudy","cards-stats","cards-insights","form"]</t>
+    <t>["cards-product","story-banner","tabs-solutions","cards-stats","cards-services","cards-news"]</t>
   </si>
   <si>
     <t>index</t>
@@ -52,13 +52,13 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-05-13T15:31:17.356Z</t>
-  </si>
-  <si>
-    <t>SEI | Financial value is created between the lines.</t>
-  </si>
-  <si>
-    <t>https://sei-demo-nextjs.vercel.app/</t>
+    <t>2026-06-18T16:53:11.414Z</t>
+  </si>
+  <si>
+    <t>The Trusted Payments and Data Company - Deluxe</t>
+  </si>
+  <si>
+    <t>https://www.deluxe.com/</t>
   </si>
 </sst>
 </file>
@@ -455,8 +455,8 @@
     <col min="3" max="3" width="7" customWidth="1"/>
     <col min="5" max="5" width="10" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="50" customWidth="1"/>
-    <col min="8" max="8" width="37" customWidth="1"/>
+    <col min="7" max="7" width="48" customWidth="1"/>
+    <col min="8" max="8" width="25" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>